<commit_message>
Initial adjustments to design following economist panel
</commit_message>
<xml_diff>
--- a/output/tables/universal_sm_hybrid/hybrid_by_route.xlsx
+++ b/output/tables/universal_sm_hybrid/hybrid_by_route.xlsx
@@ -389,19 +389,19 @@
         <v>6</v>
       </c>
       <c r="B2" t="n">
-        <v>1914</v>
+        <v>1828</v>
       </c>
       <c r="C2" t="n">
-        <v>19.4146300552779</v>
+        <v>18.4891458945881</v>
       </c>
       <c r="D2" t="n">
-        <v>42436.6793019121</v>
+        <v>41301.1279882902</v>
       </c>
       <c r="E2" t="n">
-        <v>65.2398184760953</v>
+        <v>65.7772203210134</v>
       </c>
       <c r="F2" t="n">
-        <v>10452.1104090432</v>
+        <v>9916.42468871174</v>
       </c>
     </row>
     <row r="3">
@@ -409,19 +409,19 @@
         <v>7</v>
       </c>
       <c r="B3" t="n">
-        <v>2813</v>
+        <v>2743</v>
       </c>
       <c r="C3" t="n">
-        <v>26.6521032626311</v>
+        <v>25.9833265074087</v>
       </c>
       <c r="D3" t="n">
-        <v>35452.3328727742</v>
+        <v>34767.7775508686</v>
       </c>
       <c r="E3" t="n">
-        <v>84.8234824192668</v>
+        <v>84.7042163740556</v>
       </c>
       <c r="F3" t="n">
-        <v>14470.4163753296</v>
+        <v>13949.1949654053</v>
       </c>
     </row>
   </sheetData>

</xml_diff>